<commit_message>
Added me as dev for movement + added mini map to feature tracker
</commit_message>
<xml_diff>
--- a/Feature_Tracker.xlsx
+++ b/Feature_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bdoan\source\repos\DEV2-Prototype-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8256AF-B4BC-41BC-ADE9-F9B479FEDA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B292DDB3-88F3-44EB-8898-75112DEBDCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{3D09B86F-DC8E-4082-B780-5053E8B91B87}"/>
+    <workbookView xWindow="7620" yWindow="2940" windowWidth="28800" windowHeight="15345" xr2:uid="{3D09B86F-DC8E-4082-B780-5053E8B91B87}"/>
   </bookViews>
   <sheets>
     <sheet name="Feature Tracker" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="76">
   <si>
     <t>Features</t>
   </si>
@@ -263,6 +263,12 @@
   </si>
   <si>
     <t>Map Layout</t>
+  </si>
+  <si>
+    <t>Burgy</t>
+  </si>
+  <si>
+    <t>Mini Map/ Map System</t>
   </si>
 </sst>
 </file>
@@ -658,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6B31B0D-26DC-4CBE-BC71-3F6E3D838FDE}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" customWidth="1"/>
@@ -694,6 +700,9 @@
       <c r="D2" t="s">
         <v>14</v>
       </c>
+      <c r="E2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -844,6 +853,20 @@
       </c>
       <c r="B16" s="1" t="b">
         <v>0</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>